<commit_message>
Update simulation parameters and add plotting script
Increased tray interaction mean time in agents.py and extended simulation duration in main.py. Added plotgraphs.py for visualizing queue times and introduced several new and updated Excel data files for model input and analysis.
</commit_message>
<xml_diff>
--- a/Coleta de dados Presenciais.xlsx
+++ b/Coleta de dados Presenciais.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mangu\Documents\GitHub\TrabalhoMultiDisciplinar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230A35FB-BBAD-4F01-9EE7-5A7F2807C958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A3CC4D-2210-4445-B59C-5262DF32CBA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,12 +32,11 @@
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[hh]:mm"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -49,6 +48,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -72,11 +72,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="46" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -740,6 +741,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -747,7 +749,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1580,7 +1581,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D1000"/>
+  <dimension ref="A1:N1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.5703125" customWidth="1"/>
@@ -1588,39 +1589,63 @@
     <col min="4" max="4" width="27.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="2">
         <v>0.5</v>
       </c>
       <c r="B1" s="3">
         <v>3.472222222222222E-3</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="M1" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="N1" s="3">
+        <v>2.0833333333333333E-3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>0.5</v>
       </c>
       <c r="B2" s="3">
         <v>3.5879629629629629E-3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="M2" s="4">
+        <v>0.50694444444444497</v>
+      </c>
+      <c r="N2" s="3">
+        <v>4.1666666666666666E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>0.5</v>
       </c>
       <c r="B3" s="3">
         <v>2.7777777777777779E-3</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="M3" s="4">
+        <v>0.51388888888888895</v>
+      </c>
+      <c r="N3" s="3">
+        <v>5.5555555555555558E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>0.5</v>
       </c>
       <c r="B4" s="3">
         <v>3.1250000000000002E-3</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="M4" s="4">
+        <v>0.52083333333333404</v>
+      </c>
+      <c r="N4" s="3">
+        <v>7.6388888888888886E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>0.5</v>
       </c>
@@ -1628,7 +1653,7 @@
         <v>3.7037037037037038E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>0.5</v>
       </c>
@@ -1636,7 +1661,7 @@
         <v>2.8935185185185184E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>0.5</v>
       </c>
@@ -1644,7 +1669,7 @@
         <v>3.2407407407407406E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>0.5</v>
       </c>
@@ -1652,7 +1677,7 @@
         <v>2.662037037037037E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>0.5</v>
       </c>
@@ -1660,7 +1685,7 @@
         <v>3.2407407407407406E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>0.5</v>
       </c>
@@ -1668,7 +1693,7 @@
         <v>3.1250000000000002E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>0.50694444444444442</v>
       </c>
@@ -1676,7 +1701,7 @@
         <v>7.6388888888888886E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>0.50694444444444442</v>
       </c>
@@ -1684,7 +1709,7 @@
         <v>7.060185185185185E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>0.50694444444444398</v>
       </c>
@@ -1692,7 +1717,7 @@
         <v>7.060185185185185E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>0.50694444444444398</v>
       </c>
@@ -1700,7 +1725,7 @@
         <v>7.7546296296296295E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>0.50694444444444398</v>
       </c>
@@ -1708,7 +1733,7 @@
         <v>7.4074074074074077E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>0.50694444444444398</v>
       </c>

</xml_diff>